<commit_message>
tables: refresh summary and model outputs
</commit_message>
<xml_diff>
--- a/tables/Table1_DataSummary.xlsx
+++ b/tables/Table1_DataSummary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J68"/>
+  <dimension ref="A1:J66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,7 +515,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Heard about Climate Change</t>
+          <t>Climate Change Knowledge</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -583,7 +583,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Female Dummy</t>
+          <t>Respondent Female Dummy</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -617,7 +617,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Age</t>
+          <t>Repsondent Age</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -658,10 +658,10 @@
         <v>11568</v>
       </c>
       <c r="D7" t="n">
-        <v>50.08238243430152</v>
+        <v>50.02558782849239</v>
       </c>
       <c r="E7" t="n">
-        <v>15.82942295429537</v>
+        <v>14.51367300417671</v>
       </c>
       <c r="F7" t="n">
         <v>25</v>
@@ -676,7 +676,7 @@
         <v>60</v>
       </c>
       <c r="J7" t="n">
-        <v>730</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8">
@@ -1712,10 +1712,10 @@
         <v>11568</v>
       </c>
       <c r="D38" t="n">
-        <v>0.5114972337482711</v>
+        <v>0.4447614107883817</v>
       </c>
       <c r="E38" t="n">
-        <v>0.4998894031665838</v>
+        <v>0.4969608110084769</v>
       </c>
       <c r="F38" t="n">
         <v>0</v>
@@ -1724,7 +1724,7 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I38" t="n">
         <v>1</v>
@@ -1746,10 +1746,10 @@
         <v>11568</v>
       </c>
       <c r="D39" t="n">
-        <v>0.2901970954356847</v>
+        <v>0.149896265560166</v>
       </c>
       <c r="E39" t="n">
-        <v>0.4538728335440916</v>
+        <v>0.3569851419733781</v>
       </c>
       <c r="F39" t="n">
         <v>0</v>
@@ -1761,7 +1761,7 @@
         <v>0</v>
       </c>
       <c r="I39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J39" t="n">
         <v>1</v>
@@ -1780,10 +1780,10 @@
         <v>11568</v>
       </c>
       <c r="D40" t="n">
-        <v>0.3979080221300138</v>
+        <v>0.2499135546334716</v>
       </c>
       <c r="E40" t="n">
-        <v>0.4894874259736945</v>
+        <v>0.4329814961566604</v>
       </c>
       <c r="F40" t="n">
         <v>0</v>
@@ -1795,7 +1795,7 @@
         <v>0</v>
       </c>
       <c r="I40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J40" t="n">
         <v>1</v>
@@ -1814,10 +1814,10 @@
         <v>11568</v>
       </c>
       <c r="D41" t="n">
-        <v>0.2413554633471646</v>
+        <v>0.09664591977869987</v>
       </c>
       <c r="E41" t="n">
-        <v>0.427923864062656</v>
+        <v>0.2954877895548925</v>
       </c>
       <c r="F41" t="n">
         <v>0</v>
@@ -1848,10 +1848,10 @@
         <v>11568</v>
       </c>
       <c r="D42" t="n">
-        <v>0.7568291839557399</v>
+        <v>0.9035269709543569</v>
       </c>
       <c r="E42" t="n">
-        <v>0.4290159448586778</v>
+        <v>0.2952516205869883</v>
       </c>
       <c r="F42" t="n">
         <v>0</v>
@@ -1882,10 +1882,10 @@
         <v>11568</v>
       </c>
       <c r="D43" t="n">
-        <v>0.3705048409405256</v>
+        <v>0.2576071922544951</v>
       </c>
       <c r="E43" t="n">
-        <v>0.482960834087826</v>
+        <v>0.4373354095993849</v>
       </c>
       <c r="F43" t="n">
         <v>0</v>
@@ -1916,10 +1916,10 @@
         <v>11568</v>
       </c>
       <c r="D44" t="n">
-        <v>0.2230290456431535</v>
+        <v>0.04002420470262794</v>
       </c>
       <c r="E44" t="n">
-        <v>0.4162956540774328</v>
+        <v>0.1960244613682552</v>
       </c>
       <c r="F44" t="n">
         <v>0</v>
@@ -1950,10 +1950,10 @@
         <v>11568</v>
       </c>
       <c r="D45" t="n">
-        <v>0.3739626556016598</v>
+        <v>0.3077455048409405</v>
       </c>
       <c r="E45" t="n">
-        <v>0.4838748058000238</v>
+        <v>0.4615805746013739</v>
       </c>
       <c r="F45" t="n">
         <v>0</v>
@@ -1984,10 +1984,10 @@
         <v>11568</v>
       </c>
       <c r="D46" t="n">
-        <v>0.2041839557399723</v>
+        <v>0.01910442600276625</v>
       </c>
       <c r="E46" t="n">
-        <v>0.4031214654769207</v>
+        <v>0.1368980167433992</v>
       </c>
       <c r="F46" t="n">
         <v>0</v>
@@ -2018,10 +2018,10 @@
         <v>11568</v>
       </c>
       <c r="D47" t="n">
-        <v>0.3687759336099585</v>
+        <v>0.2507780082987552</v>
       </c>
       <c r="E47" t="n">
-        <v>0.482493905571128</v>
+        <v>0.4334796908023996</v>
       </c>
       <c r="F47" t="n">
         <v>0</v>
@@ -2256,10 +2256,10 @@
         <v>11568</v>
       </c>
       <c r="D54" t="n">
-        <v>1.749818465495959</v>
+        <v>1.646084025661934</v>
       </c>
       <c r="E54" t="n">
-        <v>8.388957240239286</v>
+        <v>2.912191836669039</v>
       </c>
       <c r="F54" t="n">
         <v>0</v>
@@ -2274,7 +2274,7 @@
         <v>2</v>
       </c>
       <c r="J54" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
     </row>
     <row r="55">
@@ -2324,10 +2324,10 @@
         <v>11568</v>
       </c>
       <c r="D56" t="n">
-        <v>23.42326244813317</v>
+        <v>6.455593015214771</v>
       </c>
       <c r="E56" t="n">
-        <v>135.4055637676528</v>
+        <v>14.4270514346897</v>
       </c>
       <c r="F56" t="n">
         <v>0</v>
@@ -2342,7 +2342,7 @@
         <v>6</v>
       </c>
       <c r="J56" t="n">
-        <v>999</v>
+        <v>100</v>
       </c>
     </row>
     <row r="57">
@@ -2555,32 +2555,32 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Total Income</t>
+          <t>Survey Year</t>
         </is>
       </c>
       <c r="C63" t="n">
         <v>11568</v>
       </c>
       <c r="D63" t="n">
-        <v>323942.34906639</v>
+        <v>2019.375518672199</v>
       </c>
       <c r="E63" t="n">
-        <v>1143592.226763776</v>
+        <v>2.976533489027994</v>
       </c>
       <c r="F63" t="n">
-        <v>0</v>
+        <v>2016</v>
       </c>
       <c r="G63" t="n">
-        <v>54000</v>
+        <v>2016</v>
       </c>
       <c r="H63" t="n">
-        <v>170000</v>
+        <v>2022</v>
       </c>
       <c r="I63" t="n">
-        <v>400000</v>
+        <v>2022</v>
       </c>
       <c r="J63" t="n">
-        <v>99200000</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="64">
@@ -2589,32 +2589,32 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Survey Year</t>
+          <t>Natural Disaster Experience Indicator</t>
         </is>
       </c>
       <c r="C64" t="n">
         <v>11568</v>
       </c>
       <c r="D64" t="n">
-        <v>2019.375518672199</v>
+        <v>4.337914937759336</v>
       </c>
       <c r="E64" t="n">
-        <v>2.976533489027994</v>
+        <v>2.656074636075603</v>
       </c>
       <c r="F64" t="n">
-        <v>2016</v>
+        <v>0</v>
       </c>
       <c r="G64" t="n">
-        <v>2016</v>
+        <v>2</v>
       </c>
       <c r="H64" t="n">
-        <v>2022</v>
+        <v>4</v>
       </c>
       <c r="I64" t="n">
-        <v>2022</v>
+        <v>6</v>
       </c>
       <c r="J64" t="n">
-        <v>2022</v>
+        <v>15</v>
       </c>
     </row>
     <row r="65">
@@ -2623,32 +2623,32 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Natural Disaster Experience Indicator</t>
+          <t>Natural Disaster-related Food Shortage Indicator</t>
         </is>
       </c>
       <c r="C65" t="n">
         <v>11568</v>
       </c>
       <c r="D65" t="n">
-        <v>4.337914937759336</v>
+        <v>0.4479598893499309</v>
       </c>
       <c r="E65" t="n">
-        <v>2.656074636075603</v>
+        <v>0.9247970462074602</v>
       </c>
       <c r="F65" t="n">
         <v>0</v>
       </c>
       <c r="G65" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H65" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I65" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J65" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="66">
@@ -2657,17 +2657,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Natural Disaster-related Food Shortage Indicator</t>
+          <t>Natural Disaster-related Death Indicator</t>
         </is>
       </c>
       <c r="C66" t="n">
         <v>11568</v>
       </c>
       <c r="D66" t="n">
-        <v>0.4479598893499309</v>
+        <v>0.01045988934993084</v>
       </c>
       <c r="E66" t="n">
-        <v>0.9247970462074602</v>
+        <v>0.1042597330371103</v>
       </c>
       <c r="F66" t="n">
         <v>0</v>
@@ -2682,75 +2682,7 @@
         <v>0</v>
       </c>
       <c r="J66" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="1" t="n">
-        <v>65</v>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Natural Disaster-related Death Indicator</t>
-        </is>
-      </c>
-      <c r="C67" t="n">
-        <v>11568</v>
-      </c>
-      <c r="D67" t="n">
-        <v>0.01045988934993084</v>
-      </c>
-      <c r="E67" t="n">
-        <v>0.1042597330371103</v>
-      </c>
-      <c r="F67" t="n">
-        <v>0</v>
-      </c>
-      <c r="G67" t="n">
-        <v>0</v>
-      </c>
-      <c r="H67" t="n">
-        <v>0</v>
-      </c>
-      <c r="I67" t="n">
-        <v>0</v>
-      </c>
-      <c r="J67" t="n">
         <v>2</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="1" t="n">
-        <v>66</v>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Natural Disaster-related Loss</t>
-        </is>
-      </c>
-      <c r="C68" t="n">
-        <v>11568</v>
-      </c>
-      <c r="D68" t="n">
-        <v>0.5471991701244814</v>
-      </c>
-      <c r="E68" t="n">
-        <v>1.076411065038905</v>
-      </c>
-      <c r="F68" t="n">
-        <v>0</v>
-      </c>
-      <c r="G68" t="n">
-        <v>0</v>
-      </c>
-      <c r="H68" t="n">
-        <v>0</v>
-      </c>
-      <c r="I68" t="n">
-        <v>1</v>
-      </c>
-      <c r="J68" t="n">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>